<commit_message>
fix(bess): correct working-capital, report-tabs, and DSCR narration
Fixes three say[] lines in content/bess/videos.mjs that drifted from
docs/PRODUCT_FACTS.bess.md:
- inputs-finance: the working-capital carrying cost is increased by the WC
  Facility Fee and offset by the Late-Payment Surcharge, not the reverse
  (formula in §6.5/§10.4 has facility_fee added, LPS_rate subtracted).
- exports-reports: the Word report's Project Configuration/Technical
  Parameters/Financial Assumptions sections also draw from the Data tab
  (project type, peak-shift/grid-backup flags per §4.1), not just
  Sizing/Peak/BESS/CAPEX/OPEX/Finance.
- results-financials: DSCR min/average is reported across the debt tenor
  per §6.5, not "across the project."

Regenerated docs/bess-video-index.xlsx, which embeds the say text.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9XByuUYaNbraawLjbRNhm
</commit_message>
<xml_diff>
--- a/docs/bess-video-index.xlsx
+++ b/docs/bess-video-index.xlsx
@@ -232,7 +232,7 @@
 4. Save Project Report writes the run as a Detailed Project Report — a Word document laid out in eight sections, in a fixed order, for handing to someone who wasn't at the keyboard for the run itself.
 5. Before the numbered sections, a title page carries the logo, the report's title and subtitle, the line Detailed Project Report, D P R, the generation date, and the line Prepared with SolarLayout, BESS Project Design Solution.
 6. Section one, Executive Summary, carries a narrative paragraph and a headline table: Project IRR, Equity IRR, NPV, Total CAPEX, LCOE, LCOS, Simple Payback, MoIC.
-7. Sections two through four cover Project Configuration, Technical Parameters and Financial Assumptions — the same inputs set across the Sizing, Peak, BESS, CAPEX, OPEX and Finance tabs.
+7. Sections two through four cover Project Configuration, Technical Parameters and Financial Assumptions — the same inputs set across the Data, Sizing, Peak, BESS, CAPEX, OPEX and Finance tabs.
 8. Section five is the year-by-year Financial Results and Cash-flow table, with grid-charging columns added on any year that drew grid energy.
 9. Section six embeds the Dashboard figure as an image, when a plot exists.
 10. Section seven, Analysis and Business Recommendation, carries bulleted commentary and a bolded Recommendation verdict, based on whether the run's Project IRR meets the Project Target IRR field.
@@ -962,7 +962,7 @@
     <t xml:space="preserve">1. The Financials tab shows the same run's economics as a table: a headline block at the top, and a per-year cash-flow table beneath it.
 2. Each headline line is shown only when the model has a value to report for it.
 3. Line one: Total CAPEX, Project IRR, NPV at the Finance tab's discount rate, and the CAPEX split across Solar, Wind and BESS.
-4. Line two: Post-tax IRR, Equity IRR, WACC, and DSCR minimum and average across the project — Equity IRR and WACC only appear once debt financing is enabled.
+4. Line two: Post-tax IRR, Equity IRR, WACC, and DSCR minimum and average across the debt tenor — Equity IRR and WACC only appear once debt financing is enabled.
 5. Line three: LCOE on the basis chosen on the Finance tab, LCOS, Payback, Discounted Payback, MoIC and PI.
 6. Any individual negative figure within these lines is painted red inline.
 7. The per-year table runs one row per project year, in eight column groups: year and battery health, energy, revenue, penalty, operating cost, grid charging, working capital and replacement, and cash flow and financing.
@@ -1109,7 +1109,7 @@
 3. PPA Tariff Escalation defaults to zero per cent a year, and Terminal or Salvage Value to zero per cent of CAPEX.
 4. LCOE Energy Basis chooses the denominator the levelised cost of energy is measured against — energy delivered to load by default, or total generation, or delivered plus exported energy. The last two need an export price configured, or the model falls back to the delivered basis.
 5. Receivable Lag, the days after billing before the offtaker pays, defaults to zero, which switches the working-capital cost off entirely.
-6. When it's set above zero, Working-Capital Rate, defaulting to eleven per cent a year, prices the cost of carrying those receivables, offset by any Late-Payment Surcharge and reduced further by a facility fee.
+6. When it's set above zero, Working-Capital Rate, defaulting to eleven per cent a year, prices the cost of carrying those receivables, increased by the WC Facility Fee and offset by any Late-Payment Surcharge.
 7. Debt financing is off by default. Switching it on turns on five fields: Gearing at seventy per cent of CAPEX, Interest Rate at nine per cent, Repayment Tenor at fifteen years, Moratorium at zero years, and DSRA at zero months of debt service.
 8. Tax is off by default too. Switching it on turns on Corporate Tax Rate at twenty five point one seven per cent, MAT Rate at seventeen point one six per cent, and a depreciation method — written-down-value by default, at forty per cent a year.
 9. With both debt and tax off, results match the simple pre-tax project model.

</xml_diff>